<commit_message>
Wifi Board BOM Update.
Wifi Board ka BOM bana dia ha with price and without price.
</commit_message>
<xml_diff>
--- a/Design-Files/GTV4.0_Board/BOM/GTV4.0_Board-BOM with Price.xlsx
+++ b/Design-Files/GTV4.0_Board/BOM/GTV4.0_Board-BOM with Price.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2077" uniqueCount="1155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2262" uniqueCount="1155">
   <si>
     <t>#</t>
   </si>
@@ -3817,17 +3817,6 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3848,6 +3837,17 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4156,7 +4156,7 @@
     <col min="15" max="15" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="25.42578125" customWidth="1"/>
-    <col min="18" max="18" width="13.85546875" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="31.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4171,14 +4171,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -4258,7 +4258,9 @@
       <c r="H3" s="6" t="s">
         <v>652</v>
       </c>
-      <c r="I3" s="6"/>
+      <c r="I3" s="6" t="s">
+        <v>972</v>
+      </c>
       <c r="J3" s="6" t="s">
         <v>726</v>
       </c>
@@ -4275,7 +4277,7 @@
       <c r="N3" s="6">
         <v>65</v>
       </c>
-      <c r="O3" s="26" t="s">
+      <c r="O3" s="23" t="s">
         <v>1031</v>
       </c>
       <c r="P3" s="7">
@@ -4311,7 +4313,9 @@
       <c r="H4" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I4" s="12"/>
+      <c r="I4" s="6" t="s">
+        <v>972</v>
+      </c>
       <c r="J4" s="12" t="s">
         <v>727</v>
       </c>
@@ -4328,7 +4332,7 @@
       <c r="N4" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="O4" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P4" s="13" t="s">
@@ -4364,7 +4368,9 @@
       <c r="H5" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I5" s="6"/>
+      <c r="I5" s="6" t="s">
+        <v>972</v>
+      </c>
       <c r="J5" s="6" t="s">
         <v>728</v>
       </c>
@@ -4381,7 +4387,7 @@
       <c r="N5" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O5" s="25" t="s">
+      <c r="O5" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P5" s="7" t="s">
@@ -4417,7 +4423,9 @@
       <c r="H6" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I6" s="12"/>
+      <c r="I6" s="6" t="s">
+        <v>972</v>
+      </c>
       <c r="J6" s="12" t="s">
         <v>729</v>
       </c>
@@ -4434,7 +4442,7 @@
       <c r="N6" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O6" s="25" t="s">
+      <c r="O6" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P6" s="13" t="s">
@@ -4470,7 +4478,9 @@
       <c r="H7" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I7" s="6"/>
+      <c r="I7" s="6" t="s">
+        <v>972</v>
+      </c>
       <c r="J7" s="6" t="s">
         <v>730</v>
       </c>
@@ -4487,7 +4497,7 @@
       <c r="N7" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O7" s="25" t="s">
+      <c r="O7" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P7" s="7" t="s">
@@ -4523,7 +4533,9 @@
       <c r="H8" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I8" s="12"/>
+      <c r="I8" s="6" t="s">
+        <v>972</v>
+      </c>
       <c r="J8" s="12" t="s">
         <v>731</v>
       </c>
@@ -4540,7 +4552,7 @@
       <c r="N8" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O8" s="25" t="s">
+      <c r="O8" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P8" s="13" t="s">
@@ -4595,7 +4607,7 @@
       <c r="N9" s="6">
         <v>5</v>
       </c>
-      <c r="O9" s="25" t="s">
+      <c r="O9" s="22" t="s">
         <v>1147</v>
       </c>
       <c r="P9" s="7">
@@ -4631,7 +4643,9 @@
       <c r="H10" s="12" t="s">
         <v>655</v>
       </c>
-      <c r="I10" s="12"/>
+      <c r="I10" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J10" s="12" t="s">
         <v>732</v>
       </c>
@@ -4648,7 +4662,7 @@
       <c r="N10" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O10" s="25" t="s">
+      <c r="O10" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P10" s="13" t="s">
@@ -4684,7 +4698,9 @@
       <c r="H11" s="6" t="s">
         <v>655</v>
       </c>
-      <c r="I11" s="6"/>
+      <c r="I11" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J11" s="6" t="s">
         <v>733</v>
       </c>
@@ -4701,7 +4717,7 @@
       <c r="N11" s="6" t="s">
         <v>996</v>
       </c>
-      <c r="O11" s="25" t="s">
+      <c r="O11" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P11" s="7" t="s">
@@ -4737,7 +4753,9 @@
       <c r="H12" s="12" t="s">
         <v>656</v>
       </c>
-      <c r="I12" s="12"/>
+      <c r="I12" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J12" s="12" t="s">
         <v>978</v>
       </c>
@@ -4754,7 +4772,7 @@
       <c r="N12" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O12" s="25" t="s">
+      <c r="O12" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P12" s="13" t="s">
@@ -4790,7 +4808,9 @@
       <c r="H13" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I13" s="6"/>
+      <c r="I13" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J13" s="6" t="s">
         <v>734</v>
       </c>
@@ -4807,7 +4827,7 @@
       <c r="N13" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O13" s="25" t="s">
+      <c r="O13" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P13" s="7" t="s">
@@ -4843,7 +4863,9 @@
       <c r="H14" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I14" s="12"/>
+      <c r="I14" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J14" s="12" t="s">
         <v>735</v>
       </c>
@@ -4860,7 +4882,7 @@
       <c r="N14" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O14" s="25" t="s">
+      <c r="O14" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P14" s="13" t="s">
@@ -4896,7 +4918,9 @@
       <c r="H15" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I15" s="6"/>
+      <c r="I15" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J15" s="6" t="s">
         <v>736</v>
       </c>
@@ -4913,7 +4937,7 @@
       <c r="N15" s="6" t="s">
         <v>997</v>
       </c>
-      <c r="O15" s="25" t="s">
+      <c r="O15" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P15" s="7" t="s">
@@ -4949,7 +4973,9 @@
       <c r="H16" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I16" s="12"/>
+      <c r="I16" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J16" s="12" t="s">
         <v>737</v>
       </c>
@@ -4966,7 +4992,7 @@
       <c r="N16" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O16" s="25" t="s">
+      <c r="O16" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P16" s="13" t="s">
@@ -5002,7 +5028,9 @@
       <c r="H17" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I17" s="6"/>
+      <c r="I17" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J17" s="6" t="s">
         <v>738</v>
       </c>
@@ -5019,7 +5047,7 @@
       <c r="N17" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O17" s="25" t="s">
+      <c r="O17" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P17" s="7" t="s">
@@ -5055,7 +5083,9 @@
       <c r="H18" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I18" s="12"/>
+      <c r="I18" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J18" s="12" t="s">
         <v>739</v>
       </c>
@@ -5072,7 +5102,7 @@
       <c r="N18" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O18" s="25" t="s">
+      <c r="O18" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P18" s="13" t="s">
@@ -5108,7 +5138,9 @@
       <c r="H19" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="I19" s="6"/>
+      <c r="I19" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J19" s="6" t="s">
         <v>740</v>
       </c>
@@ -5125,7 +5157,7 @@
       <c r="N19" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O19" s="25" t="s">
+      <c r="O19" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P19" s="7" t="s">
@@ -5161,7 +5193,9 @@
       <c r="H20" s="12" t="s">
         <v>658</v>
       </c>
-      <c r="I20" s="12"/>
+      <c r="I20" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J20" s="12" t="s">
         <v>741</v>
       </c>
@@ -5178,7 +5212,7 @@
       <c r="N20" s="12" t="s">
         <v>999</v>
       </c>
-      <c r="O20" s="25" t="s">
+      <c r="O20" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P20" s="13" t="s">
@@ -5214,7 +5248,9 @@
       <c r="H21" s="6" t="s">
         <v>654</v>
       </c>
-      <c r="I21" s="6"/>
+      <c r="I21" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J21" s="6" t="s">
         <v>742</v>
       </c>
@@ -5231,7 +5267,7 @@
       <c r="N21" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O21" s="25" t="s">
+      <c r="O21" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P21" s="7" t="s">
@@ -5267,7 +5303,9 @@
       <c r="H22" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I22" s="12"/>
+      <c r="I22" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J22" s="12" t="s">
         <v>743</v>
       </c>
@@ -5284,7 +5322,7 @@
       <c r="N22" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O22" s="25" t="s">
+      <c r="O22" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P22" s="13" t="s">
@@ -5320,7 +5358,9 @@
       <c r="H23" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="I23" s="6"/>
+      <c r="I23" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J23" s="6" t="s">
         <v>744</v>
       </c>
@@ -5337,7 +5377,7 @@
       <c r="N23" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O23" s="25" t="s">
+      <c r="O23" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P23" s="7" t="s">
@@ -5373,7 +5413,9 @@
       <c r="H24" s="12" t="s">
         <v>655</v>
       </c>
-      <c r="I24" s="12"/>
+      <c r="I24" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J24" s="12" t="s">
         <v>745</v>
       </c>
@@ -5390,7 +5432,7 @@
       <c r="N24" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O24" s="25" t="s">
+      <c r="O24" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P24" s="13" t="s">
@@ -5426,7 +5468,9 @@
       <c r="H25" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="I25" s="6"/>
+      <c r="I25" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J25" s="6" t="s">
         <v>746</v>
       </c>
@@ -5443,7 +5487,7 @@
       <c r="N25" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O25" s="25" t="s">
+      <c r="O25" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P25" s="7" t="s">
@@ -5479,7 +5523,9 @@
       <c r="H26" s="12" t="s">
         <v>660</v>
       </c>
-      <c r="I26" s="12"/>
+      <c r="I26" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J26" s="12" t="s">
         <v>747</v>
       </c>
@@ -5496,7 +5542,7 @@
       <c r="N26" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O26" s="25" t="s">
+      <c r="O26" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P26" s="13" t="s">
@@ -5532,7 +5578,9 @@
       <c r="H27" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="I27" s="6"/>
+      <c r="I27" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J27" s="6" t="s">
         <v>748</v>
       </c>
@@ -5549,7 +5597,7 @@
       <c r="N27" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O27" s="25" t="s">
+      <c r="O27" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P27" s="7" t="s">
@@ -5585,7 +5633,9 @@
       <c r="H28" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I28" s="12"/>
+      <c r="I28" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J28" s="12" t="s">
         <v>749</v>
       </c>
@@ -5602,7 +5652,7 @@
       <c r="N28" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O28" s="25" t="s">
+      <c r="O28" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P28" s="13" t="s">
@@ -5638,7 +5688,9 @@
       <c r="H29" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="I29" s="6"/>
+      <c r="I29" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J29" s="6" t="s">
         <v>979</v>
       </c>
@@ -5655,7 +5707,7 @@
       <c r="N29" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O29" s="25" t="s">
+      <c r="O29" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P29" s="7" t="s">
@@ -5691,7 +5743,9 @@
       <c r="H30" s="12" t="s">
         <v>660</v>
       </c>
-      <c r="I30" s="12"/>
+      <c r="I30" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J30" s="12" t="s">
         <v>972</v>
       </c>
@@ -5708,7 +5762,7 @@
       <c r="N30" s="12">
         <v>5</v>
       </c>
-      <c r="O30" s="27" t="s">
+      <c r="O30" s="24" t="s">
         <v>1147</v>
       </c>
       <c r="P30" s="13">
@@ -5744,7 +5798,9 @@
       <c r="H31" s="6" t="s">
         <v>655</v>
       </c>
-      <c r="I31" s="6"/>
+      <c r="I31" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J31" s="6" t="s">
         <v>750</v>
       </c>
@@ -5761,7 +5817,7 @@
       <c r="N31" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O31" s="25" t="s">
+      <c r="O31" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P31" s="7" t="s">
@@ -5797,7 +5853,9 @@
       <c r="H32" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I32" s="12"/>
+      <c r="I32" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J32" s="12" t="s">
         <v>751</v>
       </c>
@@ -5814,7 +5872,7 @@
       <c r="N32" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O32" s="25" t="s">
+      <c r="O32" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P32" s="13" t="s">
@@ -5850,7 +5908,9 @@
       <c r="H33" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I33" s="6"/>
+      <c r="I33" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J33" s="6" t="s">
         <v>752</v>
       </c>
@@ -5867,7 +5927,7 @@
       <c r="N33" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O33" s="25" t="s">
+      <c r="O33" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P33" s="7" t="s">
@@ -5903,7 +5963,9 @@
       <c r="H34" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I34" s="12"/>
+      <c r="I34" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J34" s="12" t="s">
         <v>753</v>
       </c>
@@ -5920,7 +5982,7 @@
       <c r="N34" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O34" s="25" t="s">
+      <c r="O34" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P34" s="13" t="s">
@@ -5956,7 +6018,9 @@
       <c r="H35" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="I35" s="6"/>
+      <c r="I35" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J35" s="6" t="s">
         <v>754</v>
       </c>
@@ -5973,7 +6037,7 @@
       <c r="N35" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O35" s="25" t="s">
+      <c r="O35" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P35" s="7" t="s">
@@ -6009,7 +6073,9 @@
       <c r="H36" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I36" s="12"/>
+      <c r="I36" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J36" s="12" t="s">
         <v>755</v>
       </c>
@@ -6026,7 +6092,7 @@
       <c r="N36" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O36" s="25" t="s">
+      <c r="O36" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P36" s="13" t="s">
@@ -6062,7 +6128,9 @@
       <c r="H37" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I37" s="6"/>
+      <c r="I37" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J37" s="6" t="s">
         <v>756</v>
       </c>
@@ -6079,7 +6147,7 @@
       <c r="N37" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O37" s="25" t="s">
+      <c r="O37" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P37" s="7" t="s">
@@ -6115,7 +6183,9 @@
       <c r="H38" s="12" t="s">
         <v>661</v>
       </c>
-      <c r="I38" s="12"/>
+      <c r="I38" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J38" s="12" t="s">
         <v>757</v>
       </c>
@@ -6132,7 +6202,7 @@
       <c r="N38" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O38" s="25" t="s">
+      <c r="O38" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P38" s="13" t="s">
@@ -6168,7 +6238,9 @@
       <c r="H39" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I39" s="6"/>
+      <c r="I39" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J39" s="6" t="s">
         <v>758</v>
       </c>
@@ -6185,7 +6257,7 @@
       <c r="N39" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O39" s="25" t="s">
+      <c r="O39" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P39" s="7" t="s">
@@ -6221,7 +6293,9 @@
       <c r="H40" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I40" s="12"/>
+      <c r="I40" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J40" s="12" t="s">
         <v>759</v>
       </c>
@@ -6238,7 +6312,7 @@
       <c r="N40" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O40" s="25" t="s">
+      <c r="O40" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P40" s="13" t="s">
@@ -6274,7 +6348,9 @@
       <c r="H41" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="I41" s="6"/>
+      <c r="I41" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J41" s="6" t="s">
         <v>760</v>
       </c>
@@ -6291,7 +6367,7 @@
       <c r="N41" s="6" t="s">
         <v>997</v>
       </c>
-      <c r="O41" s="25" t="s">
+      <c r="O41" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P41" s="7" t="s">
@@ -6327,7 +6403,9 @@
       <c r="H42" s="12" t="s">
         <v>663</v>
       </c>
-      <c r="I42" s="12"/>
+      <c r="I42" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J42" s="12" t="s">
         <v>761</v>
       </c>
@@ -6344,7 +6422,7 @@
       <c r="N42" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O42" s="25" t="s">
+      <c r="O42" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P42" s="13" t="s">
@@ -6380,7 +6458,9 @@
       <c r="H43" s="6" t="s">
         <v>664</v>
       </c>
-      <c r="I43" s="6"/>
+      <c r="I43" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J43" s="6" t="s">
         <v>762</v>
       </c>
@@ -6397,7 +6477,7 @@
       <c r="N43" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O43" s="25" t="s">
+      <c r="O43" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P43" s="7" t="s">
@@ -6433,7 +6513,9 @@
       <c r="H44" s="12" t="s">
         <v>665</v>
       </c>
-      <c r="I44" s="12"/>
+      <c r="I44" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J44" s="12" t="s">
         <v>763</v>
       </c>
@@ -6450,7 +6532,7 @@
       <c r="N44" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O44" s="25" t="s">
+      <c r="O44" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P44" s="13" t="s">
@@ -6486,7 +6568,9 @@
       <c r="H45" s="6" t="s">
         <v>666</v>
       </c>
-      <c r="I45" s="6"/>
+      <c r="I45" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J45" s="6" t="s">
         <v>764</v>
       </c>
@@ -6503,7 +6587,7 @@
       <c r="N45" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O45" s="25" t="s">
+      <c r="O45" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P45" s="7" t="s">
@@ -6539,7 +6623,9 @@
       <c r="H46" s="12" t="s">
         <v>667</v>
       </c>
-      <c r="I46" s="12"/>
+      <c r="I46" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J46" s="12" t="s">
         <v>765</v>
       </c>
@@ -6556,7 +6642,7 @@
       <c r="N46" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O46" s="25" t="s">
+      <c r="O46" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P46" s="13" t="s">
@@ -6592,7 +6678,9 @@
       <c r="H47" s="6" t="s">
         <v>668</v>
       </c>
-      <c r="I47" s="6"/>
+      <c r="I47" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J47" s="6" t="s">
         <v>766</v>
       </c>
@@ -6609,7 +6697,7 @@
       <c r="N47" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O47" s="25" t="s">
+      <c r="O47" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P47" s="7" t="s">
@@ -6645,7 +6733,9 @@
       <c r="H48" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I48" s="12"/>
+      <c r="I48" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J48" s="12" t="s">
         <v>767</v>
       </c>
@@ -6662,7 +6752,7 @@
       <c r="N48" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O48" s="25" t="s">
+      <c r="O48" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P48" s="13" t="s">
@@ -6698,7 +6788,9 @@
       <c r="H49" s="6" t="s">
         <v>668</v>
       </c>
-      <c r="I49" s="6"/>
+      <c r="I49" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J49" s="6" t="s">
         <v>768</v>
       </c>
@@ -6715,7 +6807,7 @@
       <c r="N49" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O49" s="25" t="s">
+      <c r="O49" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P49" s="7" t="s">
@@ -6751,7 +6843,9 @@
       <c r="H50" s="12" t="s">
         <v>666</v>
       </c>
-      <c r="I50" s="12"/>
+      <c r="I50" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J50" s="12" t="s">
         <v>769</v>
       </c>
@@ -6768,7 +6862,7 @@
       <c r="N50" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O50" s="25" t="s">
+      <c r="O50" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P50" s="13" t="s">
@@ -6804,7 +6898,9 @@
       <c r="H51" s="6" t="s">
         <v>669</v>
       </c>
-      <c r="I51" s="6"/>
+      <c r="I51" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J51" s="6" t="s">
         <v>770</v>
       </c>
@@ -6821,7 +6917,7 @@
       <c r="N51" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O51" s="25" t="s">
+      <c r="O51" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P51" s="7" t="s">
@@ -6857,7 +6953,9 @@
       <c r="H52" s="12" t="s">
         <v>670</v>
       </c>
-      <c r="I52" s="12"/>
+      <c r="I52" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J52" s="12" t="s">
         <v>771</v>
       </c>
@@ -6874,7 +6972,7 @@
       <c r="N52" s="12" t="s">
         <v>1032</v>
       </c>
-      <c r="O52" s="25" t="s">
+      <c r="O52" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P52" s="13" t="s">
@@ -6910,7 +7008,9 @@
       <c r="H53" s="6" t="s">
         <v>671</v>
       </c>
-      <c r="I53" s="6"/>
+      <c r="I53" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J53" s="6" t="s">
         <v>772</v>
       </c>
@@ -6927,7 +7027,7 @@
       <c r="N53" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O53" s="25" t="s">
+      <c r="O53" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P53" s="7" t="s">
@@ -6963,7 +7063,9 @@
       <c r="H54" s="12" t="s">
         <v>672</v>
       </c>
-      <c r="I54" s="12"/>
+      <c r="I54" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J54" s="12" t="s">
         <v>773</v>
       </c>
@@ -6980,7 +7082,7 @@
       <c r="N54" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O54" s="25" t="s">
+      <c r="O54" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P54" s="13" t="s">
@@ -7016,7 +7118,9 @@
       <c r="H55" s="6" t="s">
         <v>673</v>
       </c>
-      <c r="I55" s="6"/>
+      <c r="I55" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J55" s="6" t="s">
         <v>774</v>
       </c>
@@ -7033,7 +7137,7 @@
       <c r="N55" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O55" s="25" t="s">
+      <c r="O55" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P55" s="7" t="s">
@@ -7069,7 +7173,9 @@
       <c r="H56" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I56" s="12"/>
+      <c r="I56" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J56" s="12" t="s">
         <v>775</v>
       </c>
@@ -7086,7 +7192,7 @@
       <c r="N56" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O56" s="25" t="s">
+      <c r="O56" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P56" s="13" t="s">
@@ -7122,7 +7228,9 @@
       <c r="H57" s="6" t="s">
         <v>674</v>
       </c>
-      <c r="I57" s="6"/>
+      <c r="I57" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J57" s="6" t="s">
         <v>776</v>
       </c>
@@ -7139,7 +7247,7 @@
       <c r="N57" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O57" s="25" t="s">
+      <c r="O57" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P57" s="7" t="s">
@@ -7175,7 +7283,9 @@
       <c r="H58" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I58" s="12"/>
+      <c r="I58" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J58" s="12" t="s">
         <v>777</v>
       </c>
@@ -7192,7 +7302,7 @@
       <c r="N58" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O58" s="25" t="s">
+      <c r="O58" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P58" s="13" t="s">
@@ -7228,7 +7338,9 @@
       <c r="H59" s="6" t="s">
         <v>675</v>
       </c>
-      <c r="I59" s="6"/>
+      <c r="I59" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J59" s="6" t="s">
         <v>778</v>
       </c>
@@ -7245,7 +7357,7 @@
       <c r="N59" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O59" s="25" t="s">
+      <c r="O59" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P59" s="7" t="s">
@@ -7281,7 +7393,9 @@
       <c r="H60" s="12" t="s">
         <v>676</v>
       </c>
-      <c r="I60" s="12"/>
+      <c r="I60" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J60" s="12" t="s">
         <v>779</v>
       </c>
@@ -7298,7 +7412,7 @@
       <c r="N60" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O60" s="25" t="s">
+      <c r="O60" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P60" s="13" t="s">
@@ -7334,7 +7448,9 @@
       <c r="H61" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="I61" s="6"/>
+      <c r="I61" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J61" s="6" t="s">
         <v>980</v>
       </c>
@@ -7351,7 +7467,7 @@
       <c r="N61" s="6">
         <v>45</v>
       </c>
-      <c r="O61" s="25" t="s">
+      <c r="O61" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P61" s="7">
@@ -7387,7 +7503,9 @@
       <c r="H62" s="12" t="s">
         <v>675</v>
       </c>
-      <c r="I62" s="12"/>
+      <c r="I62" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J62" s="12" t="s">
         <v>780</v>
       </c>
@@ -7404,7 +7522,7 @@
       <c r="N62" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O62" s="25" t="s">
+      <c r="O62" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P62" s="13" t="s">
@@ -7440,7 +7558,9 @@
       <c r="H63" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="I63" s="6"/>
+      <c r="I63" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J63" s="6" t="s">
         <v>981</v>
       </c>
@@ -7457,7 +7577,7 @@
       <c r="N63" s="6" t="s">
         <v>1060</v>
       </c>
-      <c r="O63" s="25" t="s">
+      <c r="O63" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P63" s="7" t="s">
@@ -7493,7 +7613,9 @@
       <c r="H64" s="12" t="s">
         <v>678</v>
       </c>
-      <c r="I64" s="12"/>
+      <c r="I64" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J64" s="12" t="s">
         <v>781</v>
       </c>
@@ -7510,7 +7632,7 @@
       <c r="N64" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O64" s="25" t="s">
+      <c r="O64" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P64" s="13" t="s">
@@ -7546,7 +7668,9 @@
       <c r="H65" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="I65" s="6"/>
+      <c r="I65" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J65" s="6" t="s">
         <v>782</v>
       </c>
@@ -7563,7 +7687,7 @@
       <c r="N65" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O65" s="25" t="s">
+      <c r="O65" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P65" s="7" t="s">
@@ -7599,7 +7723,9 @@
       <c r="H66" s="12" t="s">
         <v>679</v>
       </c>
-      <c r="I66" s="12"/>
+      <c r="I66" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J66" s="12" t="s">
         <v>783</v>
       </c>
@@ -7616,7 +7742,7 @@
       <c r="N66" s="12" t="s">
         <v>1060</v>
       </c>
-      <c r="O66" s="25" t="s">
+      <c r="O66" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P66" s="13" t="s">
@@ -7652,7 +7778,9 @@
       <c r="H67" s="6" t="s">
         <v>680</v>
       </c>
-      <c r="I67" s="6"/>
+      <c r="I67" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J67" s="6" t="s">
         <v>784</v>
       </c>
@@ -7669,7 +7797,7 @@
       <c r="N67" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O67" s="25" t="s">
+      <c r="O67" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P67" s="7" t="s">
@@ -7705,7 +7833,9 @@
       <c r="H68" s="12" t="s">
         <v>681</v>
       </c>
-      <c r="I68" s="12"/>
+      <c r="I68" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J68" s="12" t="s">
         <v>785</v>
       </c>
@@ -7722,7 +7852,7 @@
       <c r="N68" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O68" s="25" t="s">
+      <c r="O68" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P68" s="13" t="s">
@@ -7758,7 +7888,9 @@
       <c r="H69" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="I69" s="6"/>
+      <c r="I69" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J69" s="6" t="s">
         <v>786</v>
       </c>
@@ -7775,7 +7907,7 @@
       <c r="N69" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O69" s="25" t="s">
+      <c r="O69" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P69" s="7" t="s">
@@ -7811,7 +7943,9 @@
       <c r="H70" s="12" t="s">
         <v>679</v>
       </c>
-      <c r="I70" s="12"/>
+      <c r="I70" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J70" s="12" t="s">
         <v>787</v>
       </c>
@@ -7828,7 +7962,7 @@
       <c r="N70" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O70" s="25" t="s">
+      <c r="O70" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P70" s="13" t="s">
@@ -7864,7 +7998,9 @@
       <c r="H71" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="I71" s="6"/>
+      <c r="I71" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J71" s="6" t="s">
         <v>788</v>
       </c>
@@ -7881,7 +8017,7 @@
       <c r="N71" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O71" s="25" t="s">
+      <c r="O71" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P71" s="7" t="s">
@@ -7917,7 +8053,9 @@
       <c r="H72" s="12" t="s">
         <v>682</v>
       </c>
-      <c r="I72" s="12"/>
+      <c r="I72" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J72" s="12" t="s">
         <v>789</v>
       </c>
@@ -7934,7 +8072,7 @@
       <c r="N72" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O72" s="25" t="s">
+      <c r="O72" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P72" s="13" t="s">
@@ -7970,7 +8108,9 @@
       <c r="H73" s="6" t="s">
         <v>683</v>
       </c>
-      <c r="I73" s="6"/>
+      <c r="I73" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J73" s="6" t="s">
         <v>790</v>
       </c>
@@ -7987,7 +8127,7 @@
       <c r="N73" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O73" s="25" t="s">
+      <c r="O73" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P73" s="7" t="s">
@@ -8023,7 +8163,9 @@
       <c r="H74" s="12" t="s">
         <v>684</v>
       </c>
-      <c r="I74" s="12"/>
+      <c r="I74" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J74" s="12" t="s">
         <v>791</v>
       </c>
@@ -8040,7 +8182,7 @@
       <c r="N74" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O74" s="25" t="s">
+      <c r="O74" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P74" s="13" t="s">
@@ -8076,7 +8218,9 @@
       <c r="H75" s="6" t="s">
         <v>655</v>
       </c>
-      <c r="I75" s="6"/>
+      <c r="I75" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J75" s="6" t="s">
         <v>792</v>
       </c>
@@ -8093,7 +8237,7 @@
       <c r="N75" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O75" s="25" t="s">
+      <c r="O75" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P75" s="7" t="s">
@@ -8129,7 +8273,9 @@
       <c r="H76" s="12" t="s">
         <v>685</v>
       </c>
-      <c r="I76" s="12"/>
+      <c r="I76" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J76" s="12" t="s">
         <v>793</v>
       </c>
@@ -8146,7 +8292,7 @@
       <c r="N76" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O76" s="25" t="s">
+      <c r="O76" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P76" s="13" t="s">
@@ -8182,7 +8328,9 @@
       <c r="H77" s="6" t="s">
         <v>685</v>
       </c>
-      <c r="I77" s="6"/>
+      <c r="I77" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J77" s="6" t="s">
         <v>794</v>
       </c>
@@ -8199,7 +8347,7 @@
       <c r="N77" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O77" s="25" t="s">
+      <c r="O77" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P77" s="7" t="s">
@@ -8235,7 +8383,9 @@
       <c r="H78" s="12" t="s">
         <v>686</v>
       </c>
-      <c r="I78" s="12"/>
+      <c r="I78" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J78" s="12" t="s">
         <v>972</v>
       </c>
@@ -8252,7 +8402,7 @@
       <c r="N78" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O78" s="25" t="s">
+      <c r="O78" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P78" s="13" t="s">
@@ -8288,7 +8438,9 @@
       <c r="H79" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="I79" s="6"/>
+      <c r="I79" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J79" s="6" t="s">
         <v>982</v>
       </c>
@@ -8305,7 +8457,7 @@
       <c r="N79" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O79" s="25" t="s">
+      <c r="O79" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P79" s="7" t="s">
@@ -8341,7 +8493,9 @@
       <c r="H80" s="12" t="s">
         <v>687</v>
       </c>
-      <c r="I80" s="12"/>
+      <c r="I80" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J80" s="12" t="s">
         <v>972</v>
       </c>
@@ -8358,7 +8512,7 @@
       <c r="N80" s="12" t="s">
         <v>1060</v>
       </c>
-      <c r="O80" s="25" t="s">
+      <c r="O80" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P80" s="13" t="s">
@@ -8394,7 +8548,9 @@
       <c r="H81" s="6" t="s">
         <v>688</v>
       </c>
-      <c r="I81" s="6"/>
+      <c r="I81" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J81" s="6" t="s">
         <v>795</v>
       </c>
@@ -8411,7 +8567,7 @@
       <c r="N81" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O81" s="25" t="s">
+      <c r="O81" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P81" s="7" t="s">
@@ -8447,7 +8603,9 @@
       <c r="H82" s="12" t="s">
         <v>689</v>
       </c>
-      <c r="I82" s="12"/>
+      <c r="I82" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J82" s="12" t="s">
         <v>796</v>
       </c>
@@ -8464,7 +8622,7 @@
       <c r="N82" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O82" s="25" t="s">
+      <c r="O82" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P82" s="13" t="s">
@@ -8500,7 +8658,9 @@
       <c r="H83" s="6" t="s">
         <v>690</v>
       </c>
-      <c r="I83" s="6"/>
+      <c r="I83" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J83" s="6" t="s">
         <v>797</v>
       </c>
@@ -8517,7 +8677,7 @@
       <c r="N83" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O83" s="25" t="s">
+      <c r="O83" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P83" s="7" t="s">
@@ -8553,7 +8713,9 @@
       <c r="H84" s="12" t="s">
         <v>690</v>
       </c>
-      <c r="I84" s="12"/>
+      <c r="I84" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J84" s="12" t="s">
         <v>798</v>
       </c>
@@ -8570,7 +8732,7 @@
       <c r="N84" s="12">
         <v>20</v>
       </c>
-      <c r="O84" s="25" t="s">
+      <c r="O84" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P84" s="13">
@@ -8606,7 +8768,9 @@
       <c r="H85" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="I85" s="6"/>
+      <c r="I85" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J85" s="6" t="s">
         <v>799</v>
       </c>
@@ -8623,7 +8787,7 @@
       <c r="N85" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O85" s="25" t="s">
+      <c r="O85" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P85" s="7" t="s">
@@ -8678,7 +8842,7 @@
       <c r="N86" s="12" t="s">
         <v>993</v>
       </c>
-      <c r="O86" s="25" t="s">
+      <c r="O86" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P86" s="13" t="s">
@@ -8714,7 +8878,9 @@
       <c r="H87" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="I87" s="6"/>
+      <c r="I87" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J87" s="6" t="s">
         <v>800</v>
       </c>
@@ -8731,7 +8897,7 @@
       <c r="N87" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O87" s="25" t="s">
+      <c r="O87" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P87" s="7" t="s">
@@ -8767,7 +8933,9 @@
       <c r="H88" s="12" t="s">
         <v>692</v>
       </c>
-      <c r="I88" s="12"/>
+      <c r="I88" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J88" s="12" t="s">
         <v>801</v>
       </c>
@@ -8784,7 +8952,7 @@
       <c r="N88" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O88" s="25" t="s">
+      <c r="O88" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P88" s="13" t="s">
@@ -8820,7 +8988,9 @@
       <c r="H89" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="I89" s="6"/>
+      <c r="I89" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J89" s="6" t="s">
         <v>802</v>
       </c>
@@ -8837,7 +9007,7 @@
       <c r="N89" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O89" s="25" t="s">
+      <c r="O89" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P89" s="7" t="s">
@@ -8873,7 +9043,9 @@
       <c r="H90" s="12" t="s">
         <v>694</v>
       </c>
-      <c r="I90" s="12"/>
+      <c r="I90" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J90" s="12" t="s">
         <v>803</v>
       </c>
@@ -8890,7 +9062,7 @@
       <c r="N90" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O90" s="25" t="s">
+      <c r="O90" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P90" s="13" t="s">
@@ -8926,7 +9098,9 @@
       <c r="H91" s="6" t="s">
         <v>695</v>
       </c>
-      <c r="I91" s="6"/>
+      <c r="I91" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J91" s="6" t="s">
         <v>804</v>
       </c>
@@ -8943,7 +9117,7 @@
       <c r="N91" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O91" s="25" t="s">
+      <c r="O91" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P91" s="7" t="s">
@@ -8979,7 +9153,9 @@
       <c r="H92" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I92" s="12"/>
+      <c r="I92" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J92" s="12" t="s">
         <v>805</v>
       </c>
@@ -8996,7 +9172,7 @@
       <c r="N92" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O92" s="25" t="s">
+      <c r="O92" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P92" s="13" t="s">
@@ -9032,7 +9208,9 @@
       <c r="H93" s="6" t="s">
         <v>696</v>
       </c>
-      <c r="I93" s="6"/>
+      <c r="I93" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J93" s="6" t="s">
         <v>806</v>
       </c>
@@ -9079,7 +9257,9 @@
       <c r="H94" s="12" t="s">
         <v>672</v>
       </c>
-      <c r="I94" s="12"/>
+      <c r="I94" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J94" s="12" t="s">
         <v>807</v>
       </c>
@@ -9096,7 +9276,7 @@
       <c r="N94" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O94" s="25" t="s">
+      <c r="O94" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P94" s="13" t="s">
@@ -9132,7 +9312,9 @@
       <c r="H95" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="I95" s="6"/>
+      <c r="I95" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J95" s="6" t="s">
         <v>808</v>
       </c>
@@ -9149,7 +9331,7 @@
       <c r="N95" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O95" s="25" t="s">
+      <c r="O95" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P95" s="7" t="s">
@@ -9185,7 +9367,9 @@
       <c r="H96" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I96" s="12"/>
+      <c r="I96" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J96" s="12" t="s">
         <v>809</v>
       </c>
@@ -9202,7 +9386,7 @@
       <c r="N96" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O96" s="25" t="s">
+      <c r="O96" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P96" s="13" t="s">
@@ -9238,7 +9422,9 @@
       <c r="H97" s="6" t="s">
         <v>697</v>
       </c>
-      <c r="I97" s="6"/>
+      <c r="I97" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J97" s="6" t="s">
         <v>810</v>
       </c>
@@ -9255,7 +9441,7 @@
       <c r="N97" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O97" s="25" t="s">
+      <c r="O97" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P97" s="7" t="s">
@@ -9291,7 +9477,9 @@
       <c r="H98" s="12" t="s">
         <v>698</v>
       </c>
-      <c r="I98" s="12"/>
+      <c r="I98" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J98" s="12" t="s">
         <v>811</v>
       </c>
@@ -9308,7 +9496,7 @@
       <c r="N98" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O98" s="25" t="s">
+      <c r="O98" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P98" s="13" t="s">
@@ -9344,7 +9532,9 @@
       <c r="H99" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I99" s="6"/>
+      <c r="I99" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J99" s="6" t="s">
         <v>812</v>
       </c>
@@ -9361,7 +9551,7 @@
       <c r="N99" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O99" s="25" t="s">
+      <c r="O99" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P99" s="7" t="s">
@@ -9397,7 +9587,9 @@
       <c r="H100" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I100" s="12"/>
+      <c r="I100" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J100" s="12" t="s">
         <v>813</v>
       </c>
@@ -9414,7 +9606,7 @@
       <c r="N100" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O100" s="25" t="s">
+      <c r="O100" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P100" s="13" t="s">
@@ -9450,7 +9642,9 @@
       <c r="H101" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I101" s="6"/>
+      <c r="I101" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J101" s="6" t="s">
         <v>814</v>
       </c>
@@ -9467,7 +9661,7 @@
       <c r="N101" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O101" s="25" t="s">
+      <c r="O101" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P101" s="7" t="s">
@@ -9503,7 +9697,9 @@
       <c r="H102" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I102" s="12"/>
+      <c r="I102" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J102" s="12" t="s">
         <v>815</v>
       </c>
@@ -9520,7 +9716,7 @@
       <c r="N102" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O102" s="25" t="s">
+      <c r="O102" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P102" s="13" t="s">
@@ -9556,7 +9752,9 @@
       <c r="H103" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I103" s="6"/>
+      <c r="I103" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J103" s="6" t="s">
         <v>816</v>
       </c>
@@ -9573,7 +9771,7 @@
       <c r="N103" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O103" s="25" t="s">
+      <c r="O103" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P103" s="7" t="s">
@@ -9609,7 +9807,9 @@
       <c r="H104" s="12" t="s">
         <v>697</v>
       </c>
-      <c r="I104" s="12"/>
+      <c r="I104" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J104" s="12" t="s">
         <v>817</v>
       </c>
@@ -9626,7 +9826,7 @@
       <c r="N104" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O104" s="25" t="s">
+      <c r="O104" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P104" s="13" t="s">
@@ -9662,7 +9862,9 @@
       <c r="H105" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I105" s="6"/>
+      <c r="I105" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J105" s="6" t="s">
         <v>818</v>
       </c>
@@ -9679,7 +9881,7 @@
       <c r="N105" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O105" s="25" t="s">
+      <c r="O105" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P105" s="7" t="s">
@@ -9715,7 +9917,9 @@
       <c r="H106" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I106" s="12"/>
+      <c r="I106" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J106" s="12" t="s">
         <v>819</v>
       </c>
@@ -9732,7 +9936,7 @@
       <c r="N106" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O106" s="25" t="s">
+      <c r="O106" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P106" s="13" t="s">
@@ -9768,7 +9972,9 @@
       <c r="H107" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I107" s="6"/>
+      <c r="I107" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J107" s="6" t="s">
         <v>820</v>
       </c>
@@ -9785,7 +9991,7 @@
       <c r="N107" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O107" s="25" t="s">
+      <c r="O107" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P107" s="7" t="s">
@@ -9821,7 +10027,9 @@
       <c r="H108" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I108" s="12"/>
+      <c r="I108" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J108" s="12" t="s">
         <v>821</v>
       </c>
@@ -9838,7 +10046,7 @@
       <c r="N108" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O108" s="25" t="s">
+      <c r="O108" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P108" s="13" t="s">
@@ -9874,7 +10082,9 @@
       <c r="H109" s="6" t="s">
         <v>974</v>
       </c>
-      <c r="I109" s="6"/>
+      <c r="I109" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J109" s="6" t="s">
         <v>822</v>
       </c>
@@ -9891,7 +10101,7 @@
       <c r="N109" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O109" s="25" t="s">
+      <c r="O109" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P109" s="7" t="s">
@@ -9927,7 +10137,9 @@
       <c r="H110" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I110" s="12"/>
+      <c r="I110" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J110" s="12" t="s">
         <v>823</v>
       </c>
@@ -9944,7 +10156,7 @@
       <c r="N110" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O110" s="25" t="s">
+      <c r="O110" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P110" s="13" t="s">
@@ -9980,7 +10192,9 @@
       <c r="H111" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I111" s="6"/>
+      <c r="I111" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J111" s="6" t="s">
         <v>824</v>
       </c>
@@ -9997,7 +10211,7 @@
       <c r="N111" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O111" s="25" t="s">
+      <c r="O111" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P111" s="7" t="s">
@@ -10033,7 +10247,9 @@
       <c r="H112" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I112" s="12"/>
+      <c r="I112" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J112" s="12" t="s">
         <v>825</v>
       </c>
@@ -10050,7 +10266,7 @@
       <c r="N112" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O112" s="25" t="s">
+      <c r="O112" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P112" s="13" t="s">
@@ -10086,7 +10302,9 @@
       <c r="H113" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I113" s="6"/>
+      <c r="I113" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J113" s="6" t="s">
         <v>826</v>
       </c>
@@ -10103,7 +10321,7 @@
       <c r="N113" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O113" s="25" t="s">
+      <c r="O113" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P113" s="7" t="s">
@@ -10139,7 +10357,9 @@
       <c r="H114" s="17" t="s">
         <v>653</v>
       </c>
-      <c r="I114" s="17"/>
+      <c r="I114" s="18" t="s">
+        <v>972</v>
+      </c>
       <c r="J114" s="17" t="s">
         <v>827</v>
       </c>
@@ -10156,7 +10376,7 @@
       <c r="N114" s="17" t="s">
         <v>994</v>
       </c>
-      <c r="O114" s="25" t="s">
+      <c r="O114" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P114" s="18" t="s">
@@ -10193,7 +10413,9 @@
       <c r="H115" s="19" t="s">
         <v>653</v>
       </c>
-      <c r="I115" s="19"/>
+      <c r="I115" s="20" t="s">
+        <v>972</v>
+      </c>
       <c r="J115" s="19" t="s">
         <v>828</v>
       </c>
@@ -10210,7 +10432,7 @@
       <c r="N115" s="19" t="s">
         <v>994</v>
       </c>
-      <c r="O115" s="25" t="s">
+      <c r="O115" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P115" s="20" t="s">
@@ -10247,7 +10469,9 @@
       <c r="H116" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I116" s="12"/>
+      <c r="I116" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J116" s="12" t="s">
         <v>828</v>
       </c>
@@ -10264,7 +10488,7 @@
       <c r="N116" s="12" t="s">
         <v>1090</v>
       </c>
-      <c r="O116" s="25" t="s">
+      <c r="O116" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P116" s="13" t="s">
@@ -10300,7 +10524,9 @@
       <c r="H117" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I117" s="6"/>
+      <c r="I117" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J117" s="6" t="s">
         <v>829</v>
       </c>
@@ -10317,7 +10543,7 @@
       <c r="N117" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O117" s="25" t="s">
+      <c r="O117" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P117" s="7" t="s">
@@ -10353,7 +10579,9 @@
       <c r="H118" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I118" s="12"/>
+      <c r="I118" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J118" s="12" t="s">
         <v>830</v>
       </c>
@@ -10370,7 +10598,7 @@
       <c r="N118" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O118" s="25" t="s">
+      <c r="O118" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P118" s="13" t="s">
@@ -10406,7 +10634,9 @@
       <c r="H119" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I119" s="6"/>
+      <c r="I119" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J119" s="6" t="s">
         <v>831</v>
       </c>
@@ -10423,7 +10653,7 @@
       <c r="N119" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O119" s="25" t="s">
+      <c r="O119" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P119" s="7" t="s">
@@ -10459,7 +10689,9 @@
       <c r="H120" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I120" s="12"/>
+      <c r="I120" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J120" s="12" t="s">
         <v>832</v>
       </c>
@@ -10476,7 +10708,7 @@
       <c r="N120" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O120" s="25" t="s">
+      <c r="O120" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P120" s="13" t="s">
@@ -10512,7 +10744,9 @@
       <c r="H121" s="6" t="s">
         <v>699</v>
       </c>
-      <c r="I121" s="6"/>
+      <c r="I121" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J121" s="6" t="s">
         <v>833</v>
       </c>
@@ -10529,7 +10763,7 @@
       <c r="N121" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O121" s="25" t="s">
+      <c r="O121" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P121" s="7" t="s">
@@ -10565,7 +10799,9 @@
       <c r="H122" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I122" s="12"/>
+      <c r="I122" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J122" s="12" t="s">
         <v>834</v>
       </c>
@@ -10582,7 +10818,7 @@
       <c r="N122" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O122" s="25" t="s">
+      <c r="O122" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P122" s="13" t="s">
@@ -10618,7 +10854,9 @@
       <c r="H123" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I123" s="6"/>
+      <c r="I123" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J123" s="6" t="s">
         <v>835</v>
       </c>
@@ -10635,7 +10873,7 @@
       <c r="N123" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O123" s="25" t="s">
+      <c r="O123" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P123" s="7" t="s">
@@ -10671,7 +10909,9 @@
       <c r="H124" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I124" s="12"/>
+      <c r="I124" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J124" s="12" t="s">
         <v>836</v>
       </c>
@@ -10688,7 +10928,7 @@
       <c r="N124" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O124" s="25" t="s">
+      <c r="O124" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P124" s="13" t="s">
@@ -10724,7 +10964,9 @@
       <c r="H125" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I125" s="6"/>
+      <c r="I125" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J125" s="6" t="s">
         <v>837</v>
       </c>
@@ -10741,7 +10983,7 @@
       <c r="N125" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O125" s="25" t="s">
+      <c r="O125" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P125" s="7" t="s">
@@ -10777,7 +11019,9 @@
       <c r="H126" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I126" s="12"/>
+      <c r="I126" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J126" s="12" t="s">
         <v>838</v>
       </c>
@@ -10794,7 +11038,7 @@
       <c r="N126" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O126" s="25" t="s">
+      <c r="O126" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P126" s="13" t="s">
@@ -10830,7 +11074,9 @@
       <c r="H127" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I127" s="6"/>
+      <c r="I127" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J127" s="6" t="s">
         <v>839</v>
       </c>
@@ -10847,7 +11093,7 @@
       <c r="N127" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O127" s="25" t="s">
+      <c r="O127" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P127" s="7" t="s">
@@ -10883,7 +11129,9 @@
       <c r="H128" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I128" s="12"/>
+      <c r="I128" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J128" s="12" t="s">
         <v>840</v>
       </c>
@@ -10900,7 +11148,7 @@
       <c r="N128" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O128" s="25" t="s">
+      <c r="O128" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P128" s="13" t="s">
@@ -10936,7 +11184,9 @@
       <c r="H129" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I129" s="6"/>
+      <c r="I129" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J129" s="6" t="s">
         <v>841</v>
       </c>
@@ -10953,7 +11203,7 @@
       <c r="N129" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O129" s="25" t="s">
+      <c r="O129" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P129" s="7" t="s">
@@ -10989,7 +11239,9 @@
       <c r="H130" s="12" t="s">
         <v>700</v>
       </c>
-      <c r="I130" s="12"/>
+      <c r="I130" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J130" s="12" t="s">
         <v>842</v>
       </c>
@@ -11006,7 +11258,7 @@
       <c r="N130" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O130" s="25" t="s">
+      <c r="O130" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P130" s="13" t="s">
@@ -11042,7 +11294,9 @@
       <c r="H131" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I131" s="6"/>
+      <c r="I131" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J131" s="6" t="s">
         <v>843</v>
       </c>
@@ -11059,7 +11313,7 @@
       <c r="N131" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O131" s="25" t="s">
+      <c r="O131" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P131" s="7" t="s">
@@ -11095,7 +11349,9 @@
       <c r="H132" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I132" s="12"/>
+      <c r="I132" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J132" s="12" t="s">
         <v>844</v>
       </c>
@@ -11112,7 +11368,7 @@
       <c r="N132" s="12" t="s">
         <v>998</v>
       </c>
-      <c r="O132" s="25" t="s">
+      <c r="O132" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P132" s="13" t="s">
@@ -11148,7 +11404,9 @@
       <c r="H133" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I133" s="6"/>
+      <c r="I133" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J133" s="6" t="s">
         <v>845</v>
       </c>
@@ -11165,7 +11423,7 @@
       <c r="N133" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O133" s="25" t="s">
+      <c r="O133" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P133" s="7" t="s">
@@ -11201,7 +11459,9 @@
       <c r="H134" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I134" s="12"/>
+      <c r="I134" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J134" s="12" t="s">
         <v>846</v>
       </c>
@@ -11218,7 +11478,7 @@
       <c r="N134" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O134" s="25" t="s">
+      <c r="O134" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P134" s="13" t="s">
@@ -11254,7 +11514,9 @@
       <c r="H135" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I135" s="6"/>
+      <c r="I135" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J135" s="6" t="s">
         <v>847</v>
       </c>
@@ -11271,7 +11533,7 @@
       <c r="N135" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O135" s="25" t="s">
+      <c r="O135" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P135" s="7" t="s">
@@ -11307,7 +11569,9 @@
       <c r="H136" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I136" s="12"/>
+      <c r="I136" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J136" s="12" t="s">
         <v>848</v>
       </c>
@@ -11324,7 +11588,7 @@
       <c r="N136" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O136" s="25" t="s">
+      <c r="O136" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P136" s="13" t="s">
@@ -11360,7 +11624,9 @@
       <c r="H137" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I137" s="6"/>
+      <c r="I137" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J137" s="6" t="s">
         <v>849</v>
       </c>
@@ -11377,7 +11643,7 @@
       <c r="N137" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O137" s="25" t="s">
+      <c r="O137" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P137" s="7" t="s">
@@ -11413,7 +11679,9 @@
       <c r="H138" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I138" s="12"/>
+      <c r="I138" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J138" s="12" t="s">
         <v>850</v>
       </c>
@@ -11430,7 +11698,7 @@
       <c r="N138" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O138" s="25" t="s">
+      <c r="O138" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P138" s="13" t="s">
@@ -11466,7 +11734,9 @@
       <c r="H139" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I139" s="6"/>
+      <c r="I139" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J139" s="6" t="s">
         <v>851</v>
       </c>
@@ -11483,7 +11753,7 @@
       <c r="N139" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O139" s="25" t="s">
+      <c r="O139" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P139" s="7" t="s">
@@ -11519,7 +11789,9 @@
       <c r="H140" s="12" t="s">
         <v>701</v>
       </c>
-      <c r="I140" s="12"/>
+      <c r="I140" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J140" s="12" t="s">
         <v>852</v>
       </c>
@@ -11536,7 +11808,7 @@
       <c r="N140" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O140" s="25" t="s">
+      <c r="O140" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P140" s="13" t="s">
@@ -11572,7 +11844,9 @@
       <c r="H141" s="6" t="s">
         <v>702</v>
       </c>
-      <c r="I141" s="6"/>
+      <c r="I141" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J141" s="6" t="s">
         <v>983</v>
       </c>
@@ -11589,7 +11863,7 @@
       <c r="N141" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O141" s="25" t="s">
+      <c r="O141" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P141" s="7" t="s">
@@ -11625,7 +11899,9 @@
       <c r="H142" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I142" s="12"/>
+      <c r="I142" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J142" s="12" t="s">
         <v>853</v>
       </c>
@@ -11642,7 +11918,7 @@
       <c r="N142" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O142" s="25" t="s">
+      <c r="O142" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P142" s="13" t="s">
@@ -11678,7 +11954,9 @@
       <c r="H143" s="19" t="s">
         <v>653</v>
       </c>
-      <c r="I143" s="19"/>
+      <c r="I143" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J143" s="19" t="s">
         <v>984</v>
       </c>
@@ -11695,7 +11973,7 @@
       <c r="N143" s="19" t="s">
         <v>994</v>
       </c>
-      <c r="O143" s="25" t="s">
+      <c r="O143" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P143" s="20" t="s">
@@ -11732,7 +12010,9 @@
       <c r="H144" s="12" t="s">
         <v>703</v>
       </c>
-      <c r="I144" s="12"/>
+      <c r="I144" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J144" s="12" t="s">
         <v>854</v>
       </c>
@@ -11749,7 +12029,7 @@
       <c r="N144" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O144" s="25" t="s">
+      <c r="O144" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P144" s="13" t="s">
@@ -11785,7 +12065,9 @@
       <c r="H145" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I145" s="6"/>
+      <c r="I145" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J145" s="6" t="s">
         <v>984</v>
       </c>
@@ -11802,7 +12084,7 @@
       <c r="N145" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O145" s="25" t="s">
+      <c r="O145" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P145" s="7" t="s">
@@ -11838,7 +12120,9 @@
       <c r="H146" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I146" s="12"/>
+      <c r="I146" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J146" s="12" t="s">
         <v>855</v>
       </c>
@@ -11855,7 +12139,7 @@
       <c r="N146" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O146" s="25" t="s">
+      <c r="O146" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P146" s="13" t="s">
@@ -11891,7 +12175,9 @@
       <c r="H147" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I147" s="6"/>
+      <c r="I147" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J147" s="6" t="s">
         <v>856</v>
       </c>
@@ -11908,7 +12194,7 @@
       <c r="N147" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O147" s="25" t="s">
+      <c r="O147" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P147" s="7" t="s">
@@ -11944,7 +12230,9 @@
       <c r="H148" s="12" t="s">
         <v>704</v>
       </c>
-      <c r="I148" s="12"/>
+      <c r="I148" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J148" s="12" t="s">
         <v>857</v>
       </c>
@@ -11961,7 +12249,7 @@
       <c r="N148" s="12" t="s">
         <v>995</v>
       </c>
-      <c r="O148" s="25" t="s">
+      <c r="O148" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P148" s="13" t="s">
@@ -11997,7 +12285,9 @@
       <c r="H149" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I149" s="6"/>
+      <c r="I149" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J149" s="6" t="s">
         <v>858</v>
       </c>
@@ -12014,7 +12304,7 @@
       <c r="N149" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O149" s="25" t="s">
+      <c r="O149" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P149" s="7" t="s">
@@ -12050,7 +12340,9 @@
       <c r="H150" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I150" s="12"/>
+      <c r="I150" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J150" s="12" t="s">
         <v>859</v>
       </c>
@@ -12067,7 +12359,7 @@
       <c r="N150" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O150" s="25" t="s">
+      <c r="O150" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P150" s="13" t="s">
@@ -12103,7 +12395,9 @@
       <c r="H151" s="6" t="s">
         <v>702</v>
       </c>
-      <c r="I151" s="6"/>
+      <c r="I151" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J151" s="6" t="s">
         <v>985</v>
       </c>
@@ -12120,7 +12414,7 @@
       <c r="N151" s="6" t="s">
         <v>995</v>
       </c>
-      <c r="O151" s="25" t="s">
+      <c r="O151" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P151" s="7" t="s">
@@ -12156,7 +12450,9 @@
       <c r="H152" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I152" s="12"/>
+      <c r="I152" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J152" s="12" t="s">
         <v>986</v>
       </c>
@@ -12173,7 +12469,7 @@
       <c r="N152" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O152" s="25" t="s">
+      <c r="O152" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P152" s="13" t="s">
@@ -12209,7 +12505,9 @@
       <c r="H153" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I153" s="6"/>
+      <c r="I153" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J153" s="6" t="s">
         <v>860</v>
       </c>
@@ -12226,7 +12524,7 @@
       <c r="N153" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O153" s="25" t="s">
+      <c r="O153" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P153" s="7" t="s">
@@ -12262,7 +12560,9 @@
       <c r="H154" s="12" t="s">
         <v>976</v>
       </c>
-      <c r="I154" s="12"/>
+      <c r="I154" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J154" s="12" t="s">
         <v>861</v>
       </c>
@@ -12279,7 +12579,7 @@
       <c r="N154" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O154" s="25" t="s">
+      <c r="O154" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P154" s="13" t="s">
@@ -12315,7 +12615,9 @@
       <c r="H155" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I155" s="6"/>
+      <c r="I155" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J155" s="6" t="s">
         <v>862</v>
       </c>
@@ -12332,7 +12634,7 @@
       <c r="N155" s="6" t="s">
         <v>998</v>
       </c>
-      <c r="O155" s="25" t="s">
+      <c r="O155" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P155" s="7" t="s">
@@ -12368,7 +12670,9 @@
       <c r="H156" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I156" s="12"/>
+      <c r="I156" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J156" s="12" t="s">
         <v>863</v>
       </c>
@@ -12385,7 +12689,7 @@
       <c r="N156" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O156" s="25" t="s">
+      <c r="O156" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P156" s="13" t="s">
@@ -12421,7 +12725,9 @@
       <c r="H157" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I157" s="6"/>
+      <c r="I157" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J157" s="6" t="s">
         <v>864</v>
       </c>
@@ -12438,7 +12744,7 @@
       <c r="N157" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O157" s="25" t="s">
+      <c r="O157" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P157" s="7" t="s">
@@ -12474,7 +12780,9 @@
       <c r="H158" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I158" s="12"/>
+      <c r="I158" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J158" s="12" t="s">
         <v>865</v>
       </c>
@@ -12491,7 +12799,7 @@
       <c r="N158" s="12" t="s">
         <v>994</v>
       </c>
-      <c r="O158" s="25" t="s">
+      <c r="O158" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P158" s="13" t="s">
@@ -12527,7 +12835,9 @@
       <c r="H159" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="I159" s="6"/>
+      <c r="I159" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J159" s="6" t="s">
         <v>866</v>
       </c>
@@ -12544,7 +12854,7 @@
       <c r="N159" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O159" s="25" t="s">
+      <c r="O159" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P159" s="7" t="s">
@@ -12580,7 +12890,9 @@
       <c r="H160" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I160" s="12"/>
+      <c r="I160" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J160" s="12" t="s">
         <v>867</v>
       </c>
@@ -12597,7 +12909,7 @@
       <c r="N160" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O160" s="25" t="s">
+      <c r="O160" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P160" s="13" t="s">
@@ -12633,7 +12945,9 @@
       <c r="H161" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="I161" s="6"/>
+      <c r="I161" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J161" s="6" t="s">
         <v>868</v>
       </c>
@@ -12650,7 +12964,7 @@
       <c r="N161" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="O161" s="25" t="s">
+      <c r="O161" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P161" s="7" t="s">
@@ -12686,7 +13000,9 @@
       <c r="H162" s="12" t="s">
         <v>705</v>
       </c>
-      <c r="I162" s="12"/>
+      <c r="I162" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J162" s="12" t="s">
         <v>869</v>
       </c>
@@ -12703,7 +13019,7 @@
       <c r="N162" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O162" s="25" t="s">
+      <c r="O162" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P162" s="13" t="s">
@@ -12739,7 +13055,9 @@
       <c r="H163" s="6" t="s">
         <v>706</v>
       </c>
-      <c r="I163" s="6"/>
+      <c r="I163" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J163" s="6" t="s">
         <v>870</v>
       </c>
@@ -12756,7 +13074,7 @@
       <c r="N163" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O163" s="25" t="s">
+      <c r="O163" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P163" s="7" t="s">
@@ -12792,7 +13110,9 @@
       <c r="H164" s="12" t="s">
         <v>707</v>
       </c>
-      <c r="I164" s="12"/>
+      <c r="I164" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J164" s="12" t="s">
         <v>871</v>
       </c>
@@ -12809,7 +13129,7 @@
       <c r="N164" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O164" s="25" t="s">
+      <c r="O164" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P164" s="13" t="s">
@@ -12845,7 +13165,9 @@
       <c r="H165" s="6" t="s">
         <v>708</v>
       </c>
-      <c r="I165" s="6"/>
+      <c r="I165" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J165" s="6" t="s">
         <v>872</v>
       </c>
@@ -12862,7 +13184,7 @@
       <c r="N165" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O165" s="25" t="s">
+      <c r="O165" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P165" s="7" t="s">
@@ -12898,7 +13220,9 @@
       <c r="H166" s="12" t="s">
         <v>708</v>
       </c>
-      <c r="I166" s="12"/>
+      <c r="I166" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J166" s="12" t="s">
         <v>873</v>
       </c>
@@ -12915,7 +13239,7 @@
       <c r="N166" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O166" s="25" t="s">
+      <c r="O166" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P166" s="13" t="s">
@@ -12951,7 +13275,9 @@
       <c r="H167" s="6" t="s">
         <v>709</v>
       </c>
-      <c r="I167" s="6"/>
+      <c r="I167" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J167" s="6" t="s">
         <v>987</v>
       </c>
@@ -12968,7 +13294,7 @@
       <c r="N167" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O167" s="25" t="s">
+      <c r="O167" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P167" s="7" t="s">
@@ -13004,7 +13330,9 @@
       <c r="H168" s="12" t="s">
         <v>692</v>
       </c>
-      <c r="I168" s="12"/>
+      <c r="I168" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J168" s="12" t="s">
         <v>988</v>
       </c>
@@ -13021,7 +13349,7 @@
       <c r="N168" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O168" s="25" t="s">
+      <c r="O168" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P168" s="13" t="s">
@@ -13057,7 +13385,9 @@
       <c r="H169" s="6" t="s">
         <v>710</v>
       </c>
-      <c r="I169" s="6"/>
+      <c r="I169" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J169" s="6" t="s">
         <v>989</v>
       </c>
@@ -13074,7 +13404,7 @@
       <c r="N169" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O169" s="25" t="s">
+      <c r="O169" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P169" s="7" t="s">
@@ -13110,7 +13440,9 @@
       <c r="H170" s="12" t="s">
         <v>708</v>
       </c>
-      <c r="I170" s="12"/>
+      <c r="I170" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J170" s="12" t="s">
         <v>874</v>
       </c>
@@ -13127,7 +13459,7 @@
       <c r="N170" s="12" t="s">
         <v>1060</v>
       </c>
-      <c r="O170" s="25" t="s">
+      <c r="O170" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P170" s="13" t="s">
@@ -13163,7 +13495,9 @@
       <c r="H171" s="6" t="s">
         <v>711</v>
       </c>
-      <c r="I171" s="6"/>
+      <c r="I171" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J171" s="6" t="s">
         <v>875</v>
       </c>
@@ -13180,7 +13514,7 @@
       <c r="N171" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O171" s="25" t="s">
+      <c r="O171" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P171" s="7" t="s">
@@ -13216,7 +13550,9 @@
       <c r="H172" s="12" t="s">
         <v>708</v>
       </c>
-      <c r="I172" s="12"/>
+      <c r="I172" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J172" s="12" t="s">
         <v>876</v>
       </c>
@@ -13233,7 +13569,7 @@
       <c r="N172" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O172" s="25" t="s">
+      <c r="O172" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P172" s="13" t="s">
@@ -13269,7 +13605,9 @@
       <c r="H173" s="6" t="s">
         <v>708</v>
       </c>
-      <c r="I173" s="6"/>
+      <c r="I173" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J173" s="6" t="s">
         <v>877</v>
       </c>
@@ -13286,7 +13624,7 @@
       <c r="N173" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O173" s="25" t="s">
+      <c r="O173" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P173" s="7" t="s">
@@ -13322,7 +13660,9 @@
       <c r="H174" s="12" t="s">
         <v>712</v>
       </c>
-      <c r="I174" s="12"/>
+      <c r="I174" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J174" s="12" t="s">
         <v>878</v>
       </c>
@@ -13339,7 +13679,7 @@
       <c r="N174" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O174" s="25" t="s">
+      <c r="O174" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P174" s="13" t="s">
@@ -13375,7 +13715,9 @@
       <c r="H175" s="6" t="s">
         <v>708</v>
       </c>
-      <c r="I175" s="6"/>
+      <c r="I175" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J175" s="6" t="s">
         <v>879</v>
       </c>
@@ -13392,7 +13734,7 @@
       <c r="N175" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="O175" s="25" t="s">
+      <c r="O175" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P175" s="7" t="s">
@@ -13428,7 +13770,9 @@
       <c r="H176" s="12" t="s">
         <v>713</v>
       </c>
-      <c r="I176" s="12"/>
+      <c r="I176" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J176" s="12" t="s">
         <v>880</v>
       </c>
@@ -13445,7 +13789,7 @@
       <c r="N176" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O176" s="25" t="s">
+      <c r="O176" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P176" s="13" t="s">
@@ -13481,7 +13825,9 @@
       <c r="H177" s="6" t="s">
         <v>714</v>
       </c>
-      <c r="I177" s="6"/>
+      <c r="I177" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J177" s="6" t="s">
         <v>990</v>
       </c>
@@ -13498,7 +13844,7 @@
       <c r="N177" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O177" s="25" t="s">
+      <c r="O177" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P177" s="7" t="s">
@@ -13534,7 +13880,9 @@
       <c r="H178" s="12" t="s">
         <v>715</v>
       </c>
-      <c r="I178" s="12"/>
+      <c r="I178" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J178" s="12" t="s">
         <v>881</v>
       </c>
@@ -13551,7 +13899,7 @@
       <c r="N178" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O178" s="25" t="s">
+      <c r="O178" s="22" t="s">
         <v>1031</v>
       </c>
       <c r="P178" s="13" t="s">
@@ -13587,7 +13935,9 @@
       <c r="H179" s="6" t="s">
         <v>972</v>
       </c>
-      <c r="I179" s="6"/>
+      <c r="I179" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J179" s="6" t="s">
         <v>972</v>
       </c>
@@ -13604,7 +13954,7 @@
       <c r="N179" s="6">
         <v>5</v>
       </c>
-      <c r="O179" s="25" t="s">
+      <c r="O179" s="22" t="s">
         <v>1154</v>
       </c>
       <c r="P179" s="7">
@@ -13640,7 +13990,9 @@
       <c r="H180" s="12" t="s">
         <v>716</v>
       </c>
-      <c r="I180" s="12"/>
+      <c r="I180" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J180" s="12" t="s">
         <v>882</v>
       </c>
@@ -13657,7 +14009,7 @@
       <c r="N180" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O180" s="25" t="str">
+      <c r="O180" s="22" t="str">
         <f t="shared" ref="O180:O189" si="177">HYPERLINK(N180, "LCSC")</f>
         <v>LCSC</v>
       </c>
@@ -13694,7 +14046,9 @@
       <c r="H181" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="I181" s="6"/>
+      <c r="I181" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J181" s="6" t="s">
         <v>883</v>
       </c>
@@ -13711,7 +14065,7 @@
       <c r="N181" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O181" s="25" t="str">
+      <c r="O181" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -13748,7 +14102,9 @@
       <c r="H182" s="12" t="s">
         <v>717</v>
       </c>
-      <c r="I182" s="12"/>
+      <c r="I182" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J182" s="12" t="s">
         <v>884</v>
       </c>
@@ -13765,7 +14121,7 @@
       <c r="N182" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O182" s="25" t="str">
+      <c r="O182" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -13802,7 +14158,9 @@
       <c r="H183" s="6" t="s">
         <v>718</v>
       </c>
-      <c r="I183" s="6"/>
+      <c r="I183" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J183" s="6" t="s">
         <v>885</v>
       </c>
@@ -13819,7 +14177,7 @@
       <c r="N183" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O183" s="25" t="str">
+      <c r="O183" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -13856,7 +14214,9 @@
       <c r="H184" s="12" t="s">
         <v>719</v>
       </c>
-      <c r="I184" s="12"/>
+      <c r="I184" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J184" s="12" t="s">
         <v>886</v>
       </c>
@@ -13873,7 +14233,7 @@
       <c r="N184" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O184" s="25" t="str">
+      <c r="O184" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -13910,7 +14270,9 @@
       <c r="H185" s="6" t="s">
         <v>720</v>
       </c>
-      <c r="I185" s="6"/>
+      <c r="I185" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J185" s="6" t="s">
         <v>887</v>
       </c>
@@ -13927,7 +14289,7 @@
       <c r="N185" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O185" s="25" t="str">
+      <c r="O185" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -13964,7 +14326,9 @@
       <c r="H186" s="12" t="s">
         <v>721</v>
       </c>
-      <c r="I186" s="12"/>
+      <c r="I186" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J186" s="12" t="s">
         <v>888</v>
       </c>
@@ -13981,7 +14345,7 @@
       <c r="N186" s="12" t="s">
         <v>1007</v>
       </c>
-      <c r="O186" s="25" t="str">
+      <c r="O186" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -14018,7 +14382,9 @@
       <c r="H187" s="6" t="s">
         <v>722</v>
       </c>
-      <c r="I187" s="6"/>
+      <c r="I187" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J187" s="6" t="s">
         <v>889</v>
       </c>
@@ -14035,7 +14401,7 @@
       <c r="N187" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O187" s="25" t="str">
+      <c r="O187" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -14072,7 +14438,9 @@
       <c r="H188" s="12" t="s">
         <v>723</v>
       </c>
-      <c r="I188" s="12"/>
+      <c r="I188" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J188" s="12" t="s">
         <v>890</v>
       </c>
@@ -14089,7 +14457,7 @@
       <c r="N188" s="12" t="s">
         <v>992</v>
       </c>
-      <c r="O188" s="25" t="str">
+      <c r="O188" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -14126,7 +14494,9 @@
       <c r="H189" s="6" t="s">
         <v>724</v>
       </c>
-      <c r="I189" s="6"/>
+      <c r="I189" s="12" t="s">
+        <v>972</v>
+      </c>
       <c r="J189" s="6" t="s">
         <v>891</v>
       </c>
@@ -14143,7 +14513,7 @@
       <c r="N189" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="O189" s="25" t="str">
+      <c r="O189" s="22" t="str">
         <f t="shared" si="177"/>
         <v>LCSC</v>
       </c>
@@ -14158,26 +14528,26 @@
     </row>
     <row r="190" spans="1:18" ht="24.75" thickBot="1">
       <c r="A190" s="1"/>
-      <c r="B190" s="28">
+      <c r="B190" s="25">
         <f>ROW(B190)-ROW($B$2)</f>
         <v>188</v>
       </c>
-      <c r="C190" s="29" t="s">
+      <c r="C190" s="26" t="s">
         <v>1149</v>
       </c>
-      <c r="D190" s="30" t="s">
-        <v>972</v>
-      </c>
-      <c r="E190" s="31" t="s">
+      <c r="D190" s="27" t="s">
+        <v>972</v>
+      </c>
+      <c r="E190" s="28" t="s">
         <v>1150</v>
       </c>
-      <c r="F190" s="30" t="s">
-        <v>972</v>
-      </c>
-      <c r="G190" s="31" t="s">
+      <c r="F190" s="27" t="s">
+        <v>972</v>
+      </c>
+      <c r="G190" s="28" t="s">
         <v>1151</v>
       </c>
-      <c r="H190" s="30" t="s">
+      <c r="H190" s="27" t="s">
         <v>972</v>
       </c>
       <c r="I190" s="12" t="s">
@@ -14199,7 +14569,7 @@
       <c r="N190" s="6">
         <v>5</v>
       </c>
-      <c r="O190" s="25" t="s">
+      <c r="O190" s="22" t="s">
         <v>1154</v>
       </c>
       <c r="P190" s="13">
@@ -14213,26 +14583,26 @@
     </row>
     <row r="191" spans="1:18" ht="36.75" thickBot="1">
       <c r="A191" s="1"/>
-      <c r="B191" s="28">
+      <c r="B191" s="25">
         <f>ROW(B191)-ROW($B$2)</f>
         <v>189</v>
       </c>
-      <c r="C191" s="29" t="s">
+      <c r="C191" s="26" t="s">
         <v>1149</v>
       </c>
-      <c r="D191" s="30" t="s">
-        <v>972</v>
-      </c>
-      <c r="E191" s="31" t="s">
+      <c r="D191" s="27" t="s">
+        <v>972</v>
+      </c>
+      <c r="E191" s="28" t="s">
         <v>1152</v>
       </c>
-      <c r="F191" s="30" t="s">
-        <v>972</v>
-      </c>
-      <c r="G191" s="31" t="s">
+      <c r="F191" s="27" t="s">
+        <v>972</v>
+      </c>
+      <c r="G191" s="28" t="s">
         <v>1153</v>
       </c>
-      <c r="H191" s="30" t="s">
+      <c r="H191" s="27" t="s">
         <v>972</v>
       </c>
       <c r="I191" s="12" t="s">
@@ -14254,7 +14624,7 @@
       <c r="N191" s="6">
         <v>5</v>
       </c>
-      <c r="O191" s="25" t="s">
+      <c r="O191" s="22" t="s">
         <v>1154</v>
       </c>
       <c r="P191" s="7">
@@ -14280,11 +14650,11 @@
       <c r="K192" s="1"/>
       <c r="L192" s="1"/>
       <c r="M192" s="1"/>
-      <c r="N192" s="23" t="s">
+      <c r="N192" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="O192" s="24"/>
-      <c r="P192" s="24"/>
+      <c r="O192" s="31"/>
+      <c r="P192" s="31"/>
       <c r="Q192" s="10">
         <f>SUM(Q3:Q191)</f>
         <v>504.16750000000025</v>
@@ -14305,11 +14675,11 @@
       <c r="K193" s="1"/>
       <c r="L193" s="1"/>
       <c r="M193" s="1"/>
-      <c r="N193" s="23" t="s">
+      <c r="N193" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="O193" s="24"/>
-      <c r="P193" s="24"/>
+      <c r="O193" s="31"/>
+      <c r="P193" s="31"/>
       <c r="Q193" s="11">
         <f>Q192/5</f>
         <v>100.83350000000004</v>

</xml_diff>